<commit_message>
OL accruals mapping and excel files
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/ATEA.OL.xlsx
+++ b/data/obx_xlsx/ATEA.OL.xlsx
@@ -10727,7 +10727,9 @@
       <c r="R25" s="15">
         <v>194.5</v>
       </c>
-      <c r="S25" s="14"/>
+      <c r="S25" s="15">
+        <v>544.4</v>
+      </c>
       <c r="T25" s="15">
         <v>383.9</v>
       </c>

</xml_diff>